<commit_message>
data: update Gerard, HWV, Zimmerman
</commit_message>
<xml_diff>
--- a/xlsx/Gerard.xlsx
+++ b/xlsx/Gerard.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$613</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$614</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3751" uniqueCount="1565">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3758" uniqueCount="1567">
   <si>
     <t>SORT</t>
   </si>
@@ -6301,6 +6301,14 @@
     <t>1. Allegro (B-flat major) [similaire au 1er mouvement G 482]
 2. Largo (E-flat major) / Allegro (B-flat major) / Adagio (B-flat major) [fragments]
 3. Larghetto (B-flat major) [similaire au 3e mouvement G 482, avec modifications] - [Larghetto / Allegro / Presto / Larghetto]</t>
+  </si>
+  <si>
+    <t>1. Allegro comodo
+2. Adagio
+3. Allegro</t>
+  </si>
+  <si>
+    <t>[2nd version]</t>
   </si>
   <si>
     <t>G. 566</t>
@@ -7605,7 +7613,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J613"/>
+  <dimension ref="A1:J614"/>
   <sheetFormatPr defaultColWidth="8.61261261261261" defaultRowHeight="25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.61261261261261" style="1" customWidth="1"/>
@@ -22119,30 +22127,33 @@
     </row>
     <row r="600" customHeight="1" spans="1:8">
       <c r="A600" s="1">
-        <v>566</v>
+        <v>565.2</v>
       </c>
       <c r="B600" s="1" t="s">
-        <v>1535</v>
+        <v>1392</v>
       </c>
       <c r="C600" s="2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="D600" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E600" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="F600" s="3" t="s">
-        <v>1536</v>
+        <v>1535</v>
       </c>
       <c r="G600" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="H600" s="3" t="s">
+        <v>1536</v>
+      </c>
     </row>
     <row r="601" customHeight="1" spans="1:8">
       <c r="A601" s="1">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B601" s="1" t="s">
         <v>1537</v>
@@ -22165,7 +22176,7 @@
     </row>
     <row r="602" customHeight="1" spans="1:8">
       <c r="A602" s="1">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B602" s="1" t="s">
         <v>1539</v>
@@ -22188,19 +22199,19 @@
     </row>
     <row r="603" customHeight="1" spans="1:8">
       <c r="A603" s="1">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B603" s="1" t="s">
         <v>1541</v>
       </c>
       <c r="C603" s="2" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D603" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E603" s="1" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="F603" s="3" t="s">
         <v>1542</v>
@@ -22211,53 +22222,53 @@
     </row>
     <row r="604" customHeight="1" spans="1:8">
       <c r="A604" s="1">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B604" s="1" t="s">
         <v>1543</v>
       </c>
       <c r="C604" s="2" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="D604" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E604" s="1" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="F604" s="3" t="s">
         <v>1544</v>
       </c>
       <c r="G604" s="3" t="s">
-        <v>72</v>
+        <v>13</v>
       </c>
     </row>
     <row r="605" customHeight="1" spans="1:8">
       <c r="A605" s="1">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B605" s="1" t="s">
         <v>1545</v>
       </c>
       <c r="C605" s="2" t="s">
-        <v>105</v>
+        <v>47</v>
       </c>
       <c r="D605" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E605" s="1" t="s">
-        <v>106</v>
+        <v>48</v>
       </c>
       <c r="F605" s="3" t="s">
         <v>1546</v>
       </c>
       <c r="G605" s="3" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="606" ht="50" customHeight="1" spans="1:8">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="606" customHeight="1" spans="1:8">
       <c r="A606" s="1">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B606" s="1" t="s">
         <v>1547</v>
@@ -22272,7 +22283,7 @@
         <v>106</v>
       </c>
       <c r="F606" s="3" t="s">
-        <v>1546</v>
+        <v>1548</v>
       </c>
       <c r="G606" s="3" t="s">
         <v>275</v>
@@ -22280,99 +22291,99 @@
     </row>
     <row r="607" ht="50" customHeight="1" spans="1:8">
       <c r="A607" s="1">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B607" s="1" t="s">
+        <v>1549</v>
+      </c>
+      <c r="C607" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D607" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E607" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F607" s="3" t="s">
         <v>1548</v>
       </c>
-      <c r="C607" s="2" t="s">
-        <v>1331</v>
-      </c>
-      <c r="D607" s="1" t="s">
-        <v>1319</v>
-      </c>
-      <c r="E607" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F607" s="3" t="s">
-        <v>1549</v>
-      </c>
       <c r="G607" s="3" t="s">
-        <v>1550</v>
+        <v>275</v>
       </c>
     </row>
     <row r="608" ht="50" customHeight="1" spans="1:8">
       <c r="A608" s="1">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B608" s="1" t="s">
-        <v>1551</v>
+        <v>1550</v>
       </c>
       <c r="C608" s="2" t="s">
-        <v>1552</v>
+        <v>1331</v>
       </c>
       <c r="D608" s="1" t="s">
         <v>1319</v>
       </c>
       <c r="E608" s="1" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F608" s="3" t="s">
-        <v>1553</v>
+        <v>1551</v>
       </c>
       <c r="G608" s="3" t="s">
-        <v>1554</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="609" ht="50" customHeight="1" spans="1:7">
       <c r="A609" s="1">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B609" s="1" t="s">
-        <v>1555</v>
+        <v>1553</v>
       </c>
       <c r="C609" s="2" t="s">
-        <v>1327</v>
+        <v>1554</v>
       </c>
       <c r="D609" s="1" t="s">
         <v>1319</v>
       </c>
       <c r="E609" s="1" t="s">
-        <v>106</v>
+        <v>11</v>
       </c>
       <c r="F609" s="3" t="s">
+        <v>1555</v>
+      </c>
+      <c r="G609" s="3" t="s">
         <v>1556</v>
-      </c>
-      <c r="G609" s="3" t="s">
-        <v>1367</v>
       </c>
     </row>
     <row r="610" ht="50" customHeight="1" spans="1:7">
       <c r="A610" s="1">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="B610" s="1" t="s">
         <v>1557</v>
       </c>
       <c r="C610" s="2" t="s">
-        <v>297</v>
+        <v>1327</v>
       </c>
       <c r="D610" s="1" t="s">
-        <v>284</v>
+        <v>1319</v>
       </c>
       <c r="E610" s="1" t="s">
-        <v>34</v>
+        <v>106</v>
       </c>
       <c r="F610" s="3" t="s">
         <v>1558</v>
       </c>
       <c r="G610" s="3" t="s">
-        <v>286</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="611" ht="50" customHeight="1" spans="1:7">
       <c r="A611" s="1">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B611" s="1" t="s">
         <v>1559</v>
@@ -22395,42 +22406,42 @@
     </row>
     <row r="612" ht="50" customHeight="1" spans="1:7">
       <c r="A612" s="1">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B612" s="1" t="s">
         <v>1561</v>
       </c>
       <c r="C612" s="2" t="s">
-        <v>9</v>
+        <v>297</v>
       </c>
       <c r="D612" s="1" t="s">
-        <v>10</v>
+        <v>284</v>
       </c>
       <c r="E612" s="1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F612" s="3" t="s">
         <v>1562</v>
       </c>
       <c r="G612" s="3" t="s">
-        <v>13</v>
+        <v>286</v>
       </c>
     </row>
     <row r="613" ht="50" customHeight="1" spans="1:7">
       <c r="A613" s="1">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B613" s="1" t="s">
         <v>1563</v>
       </c>
       <c r="C613" s="2" t="s">
-        <v>105</v>
+        <v>9</v>
       </c>
       <c r="D613" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E613" s="1" t="s">
-        <v>106</v>
+        <v>11</v>
       </c>
       <c r="F613" s="3" t="s">
         <v>1564</v>
@@ -22439,9 +22450,32 @@
         <v>13</v>
       </c>
     </row>
+    <row r="614" ht="50" customHeight="1" spans="1:7">
+      <c r="A614" s="1">
+        <v>580</v>
+      </c>
+      <c r="B614" s="1" t="s">
+        <v>1565</v>
+      </c>
+      <c r="C614" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D614" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E614" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F614" s="3" t="s">
+        <v>1566</v>
+      </c>
+      <c r="G614" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H613" etc:filterBottomFollowUsedRange="0">
-    <sortState ref="A2:H613">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H614" etc:filterBottomFollowUsedRange="0">
+    <sortState ref="A2:H614">
       <sortCondition ref="A1"/>
     </sortState>
     <extLst/>
@@ -22526,7 +22560,7 @@
       <formula>NOT(ISERROR(SEARCH("[",C555)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C596:C613">
+  <conditionalFormatting sqref="C596:C614">
     <cfRule type="containsText" dxfId="0" priority="1" operator="between" text="[">
       <formula>NOT(ISERROR(SEARCH("[",C596)))</formula>
     </cfRule>
@@ -22544,7 +22578,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="I544:J613 I2:J523 H1:J1 A1:B1 D1:F1" evalError="1"/>
+    <ignoredError sqref="I601:J614 I544:J599 I2:J523 H1:J1 A1:B1 D1:F1" evalError="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>